<commit_message>
Worked Until SP Download File
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,28 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://appriver3651001021-my.sharepoint.com/personal/apollo_inpwrinc_com/Documents/Documents/UiPath/Time_Material_Billing/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UiPath Projects\InPwr.CoE.TimeMaterialBilling\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EED8756F-B32F-430C-BC79-CEA055CB1598}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2058FAFA-B767-4E6F-9AFB-BB5EE6A8BD7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
     <sheet name="Constants" sheetId="2" r:id="rId2"/>
     <sheet name="Assets" sheetId="3" r:id="rId3"/>
+    <sheet name="Exceptions" sheetId="4" r:id="rId4"/>
+    <sheet name="Emails" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="82">
   <si>
     <t>Name</t>
   </si>
@@ -87,19 +89,8 @@
     <t>logF_BusinessProcessName</t>
   </si>
   <si>
-    <t>Framework</t>
-  </si>
-  <si>
-    <t>Orchestrator queue Name. The value must match with the queue name defined on Orchestrator.</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
     <t>Logging field which allows grouping of log data of two or more subprocesses under the same business process name</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>OrchestratorQueueName</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>Must be 0 if working with Orchestrator queues. If &gt; 0, the robot will retry the same transaction which failed with a system exception. Must be an integer value.</t>
@@ -120,12 +111,6 @@
     <t>OrchestratorAssetFolder</t>
   </si>
   <si>
-    <t>OrchestratorQueueFolder</t>
-  </si>
-  <si>
-    <t>Folder name. The value must match a folder defined in Orchestrator and queue specified as OrchestratorQueueName should be created in this folder. For classic folders leave the value field empty.</t>
-  </si>
-  <si>
     <t>MaxConsecutiveSystemExceptions</t>
   </si>
   <si>
@@ -159,70 +144,137 @@
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
   </si>
   <si>
-    <t>ProcessABCQueue</t>
-  </si>
-  <si>
-    <t>Accepts only an Boolean (TRUE or FALSE).</t>
+    <t>ExceptionType</t>
+  </si>
+  <si>
+    <t>EmailTo</t>
+  </si>
+  <si>
+    <t>EmailBcc</t>
+  </si>
+  <si>
+    <t>EmailCc</t>
+  </si>
+  <si>
+    <t>EmailSubject</t>
+  </si>
+  <si>
+    <t>EmailBody</t>
+  </si>
+  <si>
+    <t>ExceptionCode</t>
+  </si>
+  <si>
+    <t>EXB0001</t>
+  </si>
+  <si>
+    <t>EXS0001</t>
+  </si>
+  <si>
+    <t>Business</t>
+  </si>
+  <si>
+    <t>System</t>
+  </si>
+  <si>
+    <t>Business Exception Occurred</t>
+  </si>
+  <si>
+    <t>EmailCode</t>
+  </si>
+  <si>
+    <t>SystemException Occurred</t>
+  </si>
+  <si>
+    <t>EM0001</t>
+  </si>
+  <si>
+    <t>StorageBucket Name</t>
+  </si>
+  <si>
+    <t>The name of the storage Bucket used in Process</t>
+  </si>
+  <si>
+    <t>Cred_Office365_AppID</t>
+  </si>
+  <si>
+    <t>MaxRetryInterval</t>
+  </si>
+  <si>
+    <t>MinRetryInterval</t>
+  </si>
+  <si>
+    <t>CheckAppTimeOut</t>
+  </si>
+  <si>
+    <t>DownloadTimout</t>
+  </si>
+  <si>
+    <t>Hello.
+The automation has finished processing the [&lt;JobNumber&gt;] for the Period [&lt;fromPeriod&gt;] to [&lt;toPeriod&gt;].  Please find attached the updated report.
+Please contact the automation support team with any questions you may have.
+Best regards,
+Support Team</t>
+  </si>
+  <si>
+    <t>Hello,&lt;br&gt;&lt;br&gt;Our team wanted to inform you that an exception has occurred for the following reason:&lt;br&gt;&lt;br&gt;&lt;Reason&gt;&lt;br&gt;&lt;br&gt;If you have any further questions or concerns in the meantime, please don’t hesitate to contact us.&lt;br&gt;&lt;br&gt;Thank you for your understanding.&lt;br&gt;&lt;br&gt;Best regards,&lt;br&gt;Support Team</t>
+  </si>
+  <si>
+    <t>Hello,&lt;br&gt;&lt;br&gt;Our team wanted to inform you that an exception has occurred.&lt;br&gt;&lt;br&gt;If you have any further questions or concerns in the meantime, please don’t hesitate to contact us.&lt;br&gt;&lt;br&gt;Thank you for your understanding.&lt;br&gt;&lt;br&gt;Best regards,&lt;br&gt;Support Team</t>
+  </si>
+  <si>
+    <t>32fd5246-0465-417c-bed3-518983955cb3</t>
+  </si>
+  <si>
+    <t>InPwr.Fin.TimeAndMaterialBilling</t>
+  </si>
+  <si>
+    <t>O365_Application_AssetFolder</t>
+  </si>
+  <si>
+    <t>O365_TenantId</t>
+  </si>
+  <si>
+    <t>Common Utilities</t>
+  </si>
+  <si>
+    <t>O365_Application</t>
+  </si>
+  <si>
+    <t>TimeAndMaterialBilling</t>
+  </si>
+  <si>
+    <t>calypso@inpwrinc.com;appollo@inpwrinc.com;iris@inpwrinc.com</t>
+  </si>
+  <si>
+    <t>&lt;JobNumber&gt; T&amp;MBilling_ Bot Status Report</t>
+  </si>
+  <si>
+    <t>TM_SharedDrive_MappingDriveLetter</t>
   </si>
   <si>
     <t>H</t>
   </si>
   <si>
-    <t>Drive letter should not already be mapped in the system.</t>
-  </si>
-  <si>
-    <t>&lt;DriveLetter&gt;:\RPA</t>
-  </si>
-  <si>
-    <t>\\automationsvr\automation</t>
-  </si>
-  <si>
-    <t>Actual share drive path and IP address are not allowed.</t>
-  </si>
-  <si>
-    <t>The number of retry attempts for connecting the Network share drive.</t>
-  </si>
-  <si>
-    <t>The delay or time interval before retrying the action for the Network share drive.</t>
+    <t>TM_SharedDrive_ActutalMappingPath</t>
+  </si>
+  <si>
+    <t>&lt;DriveLetter&gt;:\Automation</t>
+  </si>
+  <si>
+    <t>TM_SharedDrive_UNC</t>
+  </si>
+  <si>
+    <t>\\inpwrautomation.file.core.windows.net\automation\</t>
+  </si>
+  <si>
+    <t>TM_DriveFolderPath</t>
+  </si>
+  <si>
+    <t>&lt;DriveLetter&gt;:\RPA\TMBilling\&lt;Tenant&gt;\&lt;Job_number&gt;\MM_dd_YY</t>
   </si>
   <si>
     <t>TM_SharedDrive_MappingScript_Flag</t>
-  </si>
-  <si>
-    <t>TM_SharedDrive_MappingDriveLetter</t>
-  </si>
-  <si>
-    <t>TM_SharedDrive_ActutalMappingPath</t>
-  </si>
-  <si>
-    <t>TM_SharedDrive_UNC</t>
-  </si>
-  <si>
-    <t>TM_SharedDrive_RetryCount</t>
-  </si>
-  <si>
-    <t>TM_SharedDrive_RetryInterval</t>
-  </si>
-  <si>
-    <t>&lt;DriveLetter&gt;:\RPA\TMBilling\&lt;Tenant&gt;\MasterLog\&lt;Date&gt;</t>
-  </si>
-  <si>
-    <t>Drive Folder Path in Sharedrive</t>
-  </si>
-  <si>
-    <t>TM_DriveFolderPath</t>
-  </si>
-  <si>
-    <t>TM_OrchestratorFolderPath</t>
-  </si>
-  <si>
-    <t>TM_TimeProcessName</t>
-  </si>
-  <si>
-    <t>Billing/Time And Material Billing</t>
-  </si>
-  <si>
-    <t>InPwr.CoE.TimeBilling</t>
   </si>
 </sst>
 </file>
@@ -234,13 +286,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -261,10 +306,17 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Arial"/>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -284,34 +336,57 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{59665BD0-1A29-4A8C-897F-228E9B2A4DA2}"/>
-    <cellStyle name="Normal 3 2" xfId="2" xr:uid="{F4260CE1-08D9-4260-BAD9-3676016189CD}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -324,10 +399,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -627,13 +698,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z997"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:Z963"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" customWidth="1"/>
-    <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="3" max="3" width="81.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="43.54296875" customWidth="1"/>
+    <col min="2" max="2" width="83.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="81.453125" customWidth="1"/>
+    <col min="4" max="26" width="8.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -670,133 +741,102 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>22</v>
+    <row r="2" spans="1:26" ht="29">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
-      <c r="A3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="4" t="s">
-        <v>32</v>
+    <row r="3" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="5" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" t="s">
+        <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="30">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>23</v>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" t="s">
+        <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B7" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>45</v>
+        <v>67</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C8" t="s">
-        <v>47</v>
-      </c>
+      <c r="B8" s="14"/>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A9" t="s">
+      <c r="A9" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>47</v>
-      </c>
     </row>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A10" t="s">
-        <v>56</v>
-      </c>
-      <c r="B10" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" t="s">
-        <v>57</v>
-      </c>
-      <c r="B11" s="5">
-        <v>2</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>51</v>
+        <v>73</v>
+      </c>
+      <c r="B11" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="5">
-        <v>30</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>52</v>
+        <v>75</v>
+      </c>
+      <c r="B12" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A13" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C13" t="s">
-        <v>60</v>
+      <c r="A13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A14" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>64</v>
+      <c r="A14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" t="s">
+        <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A15" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B15" t="s">
-        <v>65</v>
+    <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A16" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="17" ht="14.25" customHeight="1"/>
     <row r="18" ht="14.25" customHeight="1"/>
     <row r="19" ht="14.25" customHeight="1"/>
@@ -1744,42 +1784,8 @@
     <row r="961" ht="14.25" customHeight="1"/>
     <row r="962" ht="14.25" customHeight="1"/>
     <row r="963" ht="14.25" customHeight="1"/>
-    <row r="964" ht="14.25" customHeight="1"/>
-    <row r="965" ht="14.25" customHeight="1"/>
-    <row r="966" ht="14.25" customHeight="1"/>
-    <row r="967" ht="14.25" customHeight="1"/>
-    <row r="968" ht="14.25" customHeight="1"/>
-    <row r="969" ht="14.25" customHeight="1"/>
-    <row r="970" ht="14.25" customHeight="1"/>
-    <row r="971" ht="14.25" customHeight="1"/>
-    <row r="972" ht="14.25" customHeight="1"/>
-    <row r="973" ht="14.25" customHeight="1"/>
-    <row r="974" ht="14.25" customHeight="1"/>
-    <row r="975" ht="14.25" customHeight="1"/>
-    <row r="976" ht="14.25" customHeight="1"/>
-    <row r="977" ht="14.25" customHeight="1"/>
-    <row r="978" ht="14.25" customHeight="1"/>
-    <row r="979" ht="14.25" customHeight="1"/>
-    <row r="980" ht="14.25" customHeight="1"/>
-    <row r="981" ht="14.25" customHeight="1"/>
-    <row r="982" ht="14.25" customHeight="1"/>
-    <row r="983" ht="14.25" customHeight="1"/>
-    <row r="984" ht="14.25" customHeight="1"/>
-    <row r="985" ht="14.25" customHeight="1"/>
-    <row r="986" ht="14.25" customHeight="1"/>
-    <row r="987" ht="14.25" customHeight="1"/>
-    <row r="988" ht="14.25" customHeight="1"/>
-    <row r="989" ht="14.25" customHeight="1"/>
-    <row r="990" ht="14.25" customHeight="1"/>
-    <row r="991" ht="14.25" customHeight="1"/>
-    <row r="992" ht="14.25" customHeight="1"/>
-    <row r="993" ht="14.25" customHeight="1"/>
-    <row r="994" ht="14.25" customHeight="1"/>
-    <row r="995" ht="14.25" customHeight="1"/>
-    <row r="996" ht="14.25" customHeight="1"/>
-    <row r="997" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="3"/>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -1788,12 +1794,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="75.453125" customWidth="1"/>
+    <col min="4" max="26" width="8.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1830,26 +1836,26 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="30">
+    <row r="2" spans="1:26" ht="29">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>25</v>
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.5">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>41</v>
+        <v>3</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1873,7 +1879,7 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -1895,7 +1901,7 @@
         <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
@@ -1906,7 +1912,7 @@
         <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
@@ -1917,62 +1923,90 @@
         <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B14">
         <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B15">
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="45">
+    <row r="17" spans="1:3" ht="29">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B17" t="b">
         <v>0</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>42</v>
+      <c r="C17" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="19" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="19" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A19" t="s">
+        <v>57</v>
+      </c>
+      <c r="B19">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20">
+        <v>15</v>
+      </c>
+    </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="22" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="22" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A22" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22">
+        <v>7</v>
+      </c>
+    </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="24" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="24" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A24" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24">
+        <v>30</v>
+      </c>
+    </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="26" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="27" spans="1:3" ht="14.25" customHeight="1"/>
@@ -2938,20 +2972,20 @@
     <row r="987" ht="14.25" customHeight="1"/>
     <row r="988" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="3"/>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:Z985"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" customWidth="1"/>
-    <col min="4" max="26" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="31.81640625" customWidth="1"/>
+    <col min="2" max="2" width="30.1796875" customWidth="1"/>
+    <col min="3" max="3" width="60.1796875" customWidth="1"/>
+    <col min="4" max="26" width="65.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -2962,7 +2996,7 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>4</v>
@@ -3974,23 +4008,363 @@
     <row r="983" ht="14.25" customHeight="1"/>
     <row r="984" ht="14.25" customHeight="1"/>
     <row r="985" ht="14.25" customHeight="1"/>
-    <row r="986" ht="14.25" customHeight="1"/>
-    <row r="987" ht="14.25" customHeight="1"/>
-    <row r="988" ht="14.25" customHeight="1"/>
-    <row r="989" ht="14.25" customHeight="1"/>
-    <row r="990" ht="14.25" customHeight="1"/>
-    <row r="991" ht="14.25" customHeight="1"/>
-    <row r="992" ht="14.25" customHeight="1"/>
-    <row r="993" ht="14.25" customHeight="1"/>
-    <row r="994" ht="14.25" customHeight="1"/>
-    <row r="995" ht="14.25" customHeight="1"/>
-    <row r="996" ht="14.25" customHeight="1"/>
-    <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
-    <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="3"/>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26A045ED-89B2-46F5-87BB-9D73B35EE197}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="18.453125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.1796875" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.1796875" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.81640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="61.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.1796875" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="18.5">
+      <c r="A1" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="72.5">
+      <c r="A2" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="58">
+      <c r="A3" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{3B0B2AFC-D37E-45B8-89FA-C16D32CAA2AB}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{720EF628-0C07-4FBE-8AF9-33943974D3CA}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F7C6B43-6EA4-4DD0-939E-D4A6AD374EA2}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="13.1796875" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.90625" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.54296875" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="72.90625" style="7" customWidth="1"/>
+    <col min="7" max="16384" width="9.1796875" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="18.5">
+      <c r="A1" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="130.5">
+      <c r="A2" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{1C8C4B7F-3CB8-4254-AE7C-56D11A73D9FD}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010048AAA657FA2D2C4E8603BA7E174CF937" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="261dd7846ccb3f53699cb3e91d1a9e22">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5f4c8a79-d716-42ba-b2af-386e98c4fa6d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="28b431a403f24d62de87b767c2aa1379" ns2:_="">
+    <xsd:import namespace="5f4c8a79-d716-42ba-b2af-386e98c4fa6d"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="5f4c8a79-d716-42ba-b2af-386e98c4fa6d" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="15" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C14F2347-1CC3-4D3D-8049-DF594CF081DD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0B2E85DE-D12E-47AD-BEA4-0EE892892E95}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33CC472E-8412-4F2C-8A3A-84648FC976FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5f4c8a79-d716-42ba-b2af-386e98c4fa6d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>